<commit_message>
added mnplus, split BOM for LenelS12 supplied parts
</commit_message>
<xml_diff>
--- a/doc/Legacy Test Fixture Documentation/Saline-Provided-M1-3200-TestFixtureDoc/BOM-M1-3200-1.xlsx
+++ b/doc/Legacy Test Fixture Documentation/Saline-Provided-M1-3200-TestFixtureDoc/BOM-M1-3200-1.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\TEST\Test Fixture Project Folders\S2\NODE_V3_M1\SLI Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\repo\newgit\m1-platform\doc\Legacy Test Fixture Documentation\Saline-Provided-M1-3200-TestFixtureDoc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07F53EF3-87F6-4106-843E-C925BF17A226}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61C3476D-A5CE-4C23-8E54-9DF1DBA2E5CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19080" yWindow="-120" windowWidth="19440" windowHeight="15000" xr2:uid="{DC0857AD-655F-47C6-91A0-009B19A543BF}"/>
+    <workbookView xWindow="7580" yWindow="3060" windowWidth="28800" windowHeight="15360" xr2:uid="{DC0857AD-655F-47C6-91A0-009B19A543BF}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="M1-3200 Saline BOM Purchase" sheetId="1" r:id="rId1"/>
+    <sheet name="LenelS2 Supplied Items" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="241">
   <si>
     <t>Description</t>
   </si>
@@ -365,9 +366,6 @@
     <t>5454935-ND</t>
   </si>
   <si>
-    <t>Flash drive, 128GB</t>
-  </si>
-  <si>
     <t>Ethernet cable, Cat5e, 1 ft.</t>
   </si>
   <si>
@@ -449,9 +447,6 @@
     <t>61117-2</t>
   </si>
   <si>
-    <t>FTDI, Future Technology Devices</t>
-  </si>
-  <si>
     <t>0346-1.000-E-T</t>
   </si>
   <si>
@@ -509,15 +504,6 @@
     <t>USB cabel, micro to A, 1ft.</t>
   </si>
   <si>
-    <t>USB to TTL 5V Serial cable</t>
-  </si>
-  <si>
-    <t>768-1323-ND</t>
-  </si>
-  <si>
-    <t>TTL-232X-5V</t>
-  </si>
-  <si>
     <t>Ethernet connector, panel mount</t>
   </si>
   <si>
@@ -575,9 +561,6 @@
     <t>S2</t>
   </si>
   <si>
-    <t>S2 Test PWA</t>
-  </si>
-  <si>
     <t>SAM-E PWA</t>
   </si>
   <si>
@@ -590,15 +573,6 @@
     <t>Drawing No. BOM-M1-3200-1</t>
   </si>
   <si>
-    <t>Kingston Technology</t>
-  </si>
-  <si>
-    <t>DTXM/128GBBK</t>
-  </si>
-  <si>
-    <t>5297-DTXM/128GBBK-ND</t>
-  </si>
-  <si>
     <t>USB to CBL cable, 300mm</t>
   </si>
   <si>
@@ -684,13 +658,118 @@
   </si>
   <si>
     <t>M1-3200 Test Fixture BOM</t>
+  </si>
+  <si>
+    <t>LeneS2</t>
+  </si>
+  <si>
+    <t>LenelS2 M1-3200 test board Test PWA</t>
+  </si>
+  <si>
+    <t>LenelS2 ACM (aka mercury test board) test board Test PWA</t>
+  </si>
+  <si>
+    <t>M1-3200 Test fixture PWA</t>
+  </si>
+  <si>
+    <t>ACM test board</t>
+  </si>
+  <si>
+    <t>Fanless test fixture PC, Intel Atom or better, 4 GB RAM minimum, 128 GB storage minimum</t>
+  </si>
+  <si>
+    <t>TBD</t>
+  </si>
+  <si>
+    <t>LenelS2</t>
+  </si>
+  <si>
+    <t>Wireless thermal label printer, USB and Wi-Fi, 300 dpi, up to 110 labels/minute, black and red printing</t>
+  </si>
+  <si>
+    <t>Brother</t>
+  </si>
+  <si>
+    <t>QL-810WC</t>
+  </si>
+  <si>
+    <t>MNPlus Add-ins Test Fixture BOM</t>
+  </si>
+  <si>
+    <t>Mean Well IRM-60-48ST AC to DC Power Supply</t>
+  </si>
+  <si>
+    <t>Meanwell</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> IRM-60-48ST</t>
+  </si>
+  <si>
+    <t>Relay Board for Raspberry Arduino Relay Module 1 Channel Opto-Isolated High or Low Level Trigger (12V)</t>
+  </si>
+  <si>
+    <t>ACEIRMC</t>
+  </si>
+  <si>
+    <t>Systems POE-INJ-1000-WT High PoE 4 Pair Injector</t>
+  </si>
+  <si>
+    <t>TYCON SYSTEMS, INC</t>
+  </si>
+  <si>
+    <t>POE-INJ-1000-WT</t>
+  </si>
+  <si>
+    <t>UGREEN 2 Pack USB Extension Cable (3 FT+ 3 FT), Nylon Braided Extender Compatible With Webcam, Camera, Phone, Hub, Mouse, Keyboard, Printer, Hard Drive, Headset</t>
+  </si>
+  <si>
+    <t>UGREEN GROUP LIMITED</t>
+  </si>
+  <si>
+    <t>10495P</t>
+  </si>
+  <si>
+    <t>Acer SD Card Reader, USB A 3.0 to Micro Memory Card Reader Aluminum | Dual Slot SD to USB Adapter for Computer, PC, Laptop and Type A Devices, Compatible with SD/Micro SDXC/SDXC/SDHC/MMC/TF Cards</t>
+  </si>
+  <si>
+    <t>Acer</t>
+  </si>
+  <si>
+    <t>ODK550</t>
+  </si>
+  <si>
+    <t>PNY 32GB Elite Class 10 U1 V10 SDHC Flash Memory Card - 100MB/s Read, Class 10, U1 Full HD, UHS-I, Full Size SD</t>
+  </si>
+  <si>
+    <t>PNY</t>
+  </si>
+  <si>
+    <t>SD32GX5U1100EL-MP</t>
+  </si>
+  <si>
+    <t>DTECH 3ft USB to TTL Serial Cable 3.3V 6 Pin UART Adapter Genuine FTDI FT232RL Chip Debug Cord Compatible with Windows 11 10 8 7 Linux MAC OS 6Pin 3v3 Level Signal 2.54mm Dupont Female Header</t>
+  </si>
+  <si>
+    <t>DTECH</t>
+  </si>
+  <si>
+    <t>DT-6554-1.0M</t>
+  </si>
+  <si>
+    <t>Estimated M1-3200 total:</t>
+  </si>
+  <si>
+    <t>Estimated MNPlus  total:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
+  </numFmts>
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -726,6 +805,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -753,7 +838,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -781,6 +866,18 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="6" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1116,33 +1213,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A289F17D-22C8-41D1-9CDC-45192CD72901}">
-  <dimension ref="A1:F77"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F75"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="37.140625" customWidth="1"/>
-    <col min="2" max="2" width="10.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.140625" customWidth="1"/>
-    <col min="4" max="4" width="20.140625" customWidth="1"/>
-    <col min="5" max="5" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.28515625" customWidth="1"/>
+    <col min="1" max="1" width="37.1796875" customWidth="1"/>
+    <col min="2" max="2" width="10.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.1796875" customWidth="1"/>
+    <col min="4" max="4" width="20.1796875" customWidth="1"/>
+    <col min="5" max="5" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -1162,7 +1259,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -1182,7 +1279,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1202,7 +1299,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -1213,18 +1310,18 @@
         <v>5</v>
       </c>
       <c r="D7" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E7" t="s">
         <v>5</v>
       </c>
       <c r="F7" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>138</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>140</v>
       </c>
       <c r="B8" s="1">
         <v>2</v>
@@ -1233,16 +1330,16 @@
         <v>5</v>
       </c>
       <c r="D8" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E8" t="s">
         <v>5</v>
       </c>
       <c r="F8" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -1259,7 +1356,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>43</v>
       </c>
@@ -1279,7 +1376,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>14</v>
       </c>
@@ -1299,7 +1396,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>44</v>
       </c>
@@ -1319,7 +1416,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>18</v>
       </c>
@@ -1339,7 +1436,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>85</v>
       </c>
@@ -1347,19 +1444,19 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D14" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E14" t="s">
         <v>58</v>
       </c>
       <c r="F14" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>86</v>
       </c>
@@ -1367,19 +1464,19 @@
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E15" t="s">
         <v>58</v>
       </c>
       <c r="F15" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>79</v>
       </c>
@@ -1399,7 +1496,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
         <v>19</v>
       </c>
@@ -1419,7 +1516,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>57</v>
       </c>
@@ -1439,47 +1536,47 @@
         <v>59</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
+        <v>117</v>
+      </c>
+      <c r="B19" s="1">
+        <v>1</v>
+      </c>
+      <c r="C19" t="s">
         <v>118</v>
       </c>
-      <c r="B19" s="1">
-        <v>1</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="D19" s="8" t="s">
         <v>119</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>120</v>
       </c>
       <c r="E19" t="s">
         <v>27</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B20" s="1">
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D20" s="4">
         <v>29926</v>
       </c>
       <c r="E20" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F20" s="4">
         <v>29926</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
         <v>35</v>
       </c>
@@ -1499,7 +1596,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>40</v>
       </c>
@@ -1519,9 +1616,9 @@
         <v>37</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="B23" s="1">
         <v>1</v>
@@ -1539,349 +1636,349 @@
         <v>103</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>109</v>
-      </c>
-      <c r="B24" s="1">
-        <v>1</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>184</v>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C24" t="s">
+        <v>114</v>
       </c>
       <c r="D24" t="s">
-        <v>185</v>
+        <v>115</v>
       </c>
       <c r="E24" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="F24" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
-        <v>21</v>
+        <v>116</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>20</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>56</v>
       </c>
       <c r="C25" t="s">
-        <v>115</v>
-      </c>
-      <c r="D25" t="s">
-        <v>116</v>
+        <v>28</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>29</v>
       </c>
       <c r="E25" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="F25" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>56</v>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26" s="1">
+        <v>3</v>
       </c>
       <c r="C26" t="s">
-        <v>28</v>
-      </c>
-      <c r="D26" s="8" t="s">
-        <v>29</v>
+        <v>45</v>
+      </c>
+      <c r="D26" s="4">
+        <v>3015393</v>
       </c>
       <c r="E26" t="s">
-        <v>27</v>
-      </c>
-      <c r="F26" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+      <c r="F26" s="4">
+        <v>3015393</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
-        <v>46</v>
+        <v>25</v>
       </c>
       <c r="B27" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C27" t="s">
-        <v>45</v>
-      </c>
-      <c r="D27" s="4">
-        <v>3015393</v>
+        <v>30</v>
+      </c>
+      <c r="D27" t="s">
+        <v>132</v>
       </c>
       <c r="E27" t="s">
-        <v>45</v>
-      </c>
-      <c r="F27" s="4">
-        <v>3015393</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
-        <v>25</v>
+        <v>30</v>
+      </c>
+      <c r="F27" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>22</v>
       </c>
       <c r="B28" s="1">
         <v>2</v>
       </c>
       <c r="C28" t="s">
-        <v>30</v>
-      </c>
-      <c r="D28" t="s">
-        <v>133</v>
+        <v>139</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>140</v>
       </c>
       <c r="E28" t="s">
-        <v>30</v>
-      </c>
-      <c r="F28" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>22</v>
       </c>
       <c r="B29" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C29" t="s">
-        <v>141</v>
+        <v>76</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>142</v>
+        <v>121</v>
       </c>
       <c r="E29" t="s">
         <v>27</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>22</v>
-      </c>
-      <c r="B30" s="1">
-        <v>4</v>
+        <v>122</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A30" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>142</v>
       </c>
       <c r="C30" t="s">
-        <v>76</v>
+        <v>123</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E30" t="s">
         <v>27</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
-        <v>23</v>
+        <v>125</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>98</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>144</v>
+        <v>99</v>
       </c>
       <c r="C31" t="s">
-        <v>124</v>
+        <v>30</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>125</v>
+        <v>97</v>
       </c>
       <c r="E31" t="s">
+        <v>30</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="B32" s="1">
+        <v>1</v>
+      </c>
+      <c r="C32" t="s">
+        <v>30</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="E32" t="s">
+        <v>30</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>24</v>
+      </c>
+      <c r="B33" s="1">
+        <v>1</v>
+      </c>
+      <c r="C33" t="s">
+        <v>106</v>
+      </c>
+      <c r="D33" s="9">
+        <v>8029</v>
+      </c>
+      <c r="E33" t="s">
+        <v>58</v>
+      </c>
+      <c r="F33" s="10" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="B34" s="1">
+        <v>1</v>
+      </c>
+      <c r="C34" t="s">
+        <v>110</v>
+      </c>
+      <c r="D34" s="10">
+        <v>54171</v>
+      </c>
+      <c r="E34" t="s">
+        <v>110</v>
+      </c>
+      <c r="F34" s="4">
+        <v>54171</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B35" s="1">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>110</v>
+      </c>
+      <c r="D35" s="10">
+        <v>27423</v>
+      </c>
+      <c r="E35" t="s">
+        <v>110</v>
+      </c>
+      <c r="F35" s="5">
+        <v>27423</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>178</v>
+      </c>
+      <c r="B36" s="1">
+        <v>1</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="E36" t="s">
+        <v>58</v>
+      </c>
+      <c r="F36" s="12" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>109</v>
+      </c>
+      <c r="B37" s="1">
+        <v>1</v>
+      </c>
+      <c r="C37" t="s">
+        <v>110</v>
+      </c>
+      <c r="D37" s="4">
+        <v>23828</v>
+      </c>
+      <c r="E37" t="s">
+        <v>110</v>
+      </c>
+      <c r="F37" s="4">
+        <v>23828</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>111</v>
+      </c>
+      <c r="B38" s="1">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>110</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="E38" t="s">
+        <v>110</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A39" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C39" t="s">
+        <v>47</v>
+      </c>
+      <c r="D39" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="E39" t="s">
         <v>27</v>
       </c>
-      <c r="F31" s="8" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>98</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="C32" t="s">
-        <v>30</v>
-      </c>
-      <c r="D32" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="E32" t="s">
-        <v>30</v>
-      </c>
-      <c r="F32" s="8" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="B33" s="1">
-        <v>1</v>
-      </c>
-      <c r="C33" t="s">
-        <v>30</v>
-      </c>
-      <c r="D33" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="E33" t="s">
-        <v>30</v>
-      </c>
-      <c r="F33" s="8" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>24</v>
-      </c>
-      <c r="B34" s="1">
-        <v>1</v>
-      </c>
-      <c r="C34" t="s">
-        <v>106</v>
-      </c>
-      <c r="D34" s="9">
-        <v>8029</v>
-      </c>
-      <c r="E34" t="s">
-        <v>58</v>
-      </c>
-      <c r="F34" s="10" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="B35" s="1">
-        <v>1</v>
-      </c>
-      <c r="C35" t="s">
-        <v>111</v>
-      </c>
-      <c r="D35" s="10">
-        <v>54171</v>
-      </c>
-      <c r="E35" t="s">
-        <v>111</v>
-      </c>
-      <c r="F35" s="4">
-        <v>54171</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="B36" s="1">
-        <v>1</v>
-      </c>
-      <c r="C36" t="s">
-        <v>111</v>
-      </c>
-      <c r="D36" s="10">
-        <v>27423</v>
-      </c>
-      <c r="E36" t="s">
-        <v>111</v>
-      </c>
-      <c r="F36" s="5">
-        <v>27423</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>157</v>
-      </c>
-      <c r="B37" s="1">
-        <v>1</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D37" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="E37" t="s">
-        <v>58</v>
-      </c>
-      <c r="F37" s="12" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>187</v>
-      </c>
-      <c r="B38" s="1">
-        <v>1</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="D38" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="E38" t="s">
-        <v>58</v>
-      </c>
-      <c r="F38" s="12" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>110</v>
-      </c>
-      <c r="B39" s="1">
-        <v>1</v>
-      </c>
-      <c r="C39" t="s">
-        <v>111</v>
-      </c>
-      <c r="D39" s="4">
-        <v>23828</v>
-      </c>
-      <c r="E39" t="s">
-        <v>111</v>
-      </c>
-      <c r="F39" s="4">
-        <v>23828</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>112</v>
-      </c>
-      <c r="B40" s="1">
-        <v>1</v>
+      <c r="F39" s="8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A40" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>56</v>
       </c>
       <c r="C40" t="s">
-        <v>111</v>
-      </c>
-      <c r="D40" s="6" t="s">
-        <v>113</v>
+        <v>47</v>
+      </c>
+      <c r="D40" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="E40" t="s">
-        <v>111</v>
-      </c>
-      <c r="F40" s="6" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+      <c r="F40" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>56</v>
@@ -1890,18 +1987,18 @@
         <v>47</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="E41" t="s">
         <v>27</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>56</v>
@@ -1910,96 +2007,96 @@
         <v>47</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E42" t="s">
         <v>27</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>56</v>
+        <v>201</v>
       </c>
       <c r="C43" t="s">
         <v>47</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>48</v>
+        <v>202</v>
       </c>
       <c r="E43" t="s">
         <v>27</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" s="3" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>56</v>
       </c>
       <c r="C44" t="s">
-        <v>47</v>
+        <v>197</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>50</v>
+        <v>198</v>
       </c>
       <c r="E44" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="F44" s="8" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>210</v>
+        <v>199</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>81</v>
+      </c>
+      <c r="B45" s="1">
+        <v>1</v>
       </c>
       <c r="C45" t="s">
-        <v>47</v>
-      </c>
-      <c r="D45" s="8" t="s">
-        <v>211</v>
+        <v>82</v>
+      </c>
+      <c r="D45" s="7" t="s">
+        <v>83</v>
       </c>
       <c r="E45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F45" s="8" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
+      </c>
+      <c r="F45" s="7" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>81</v>
+      </c>
+      <c r="B46" s="1">
+        <v>1</v>
       </c>
       <c r="C46" t="s">
-        <v>206</v>
-      </c>
-      <c r="D46" s="8" t="s">
-        <v>207</v>
+        <v>104</v>
+      </c>
+      <c r="D46" s="10">
+        <v>5454948</v>
       </c>
       <c r="E46" t="s">
         <v>58</v>
       </c>
-      <c r="F46" s="8" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F46" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>81</v>
       </c>
@@ -2007,179 +2104,179 @@
         <v>1</v>
       </c>
       <c r="C47" t="s">
-        <v>82</v>
-      </c>
-      <c r="D47" s="7" t="s">
-        <v>83</v>
+        <v>104</v>
+      </c>
+      <c r="D47" s="9">
+        <v>5454935</v>
       </c>
       <c r="E47" t="s">
         <v>58</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B48" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C48" t="s">
-        <v>104</v>
-      </c>
-      <c r="D48" s="10">
-        <v>5454948</v>
+        <v>76</v>
+      </c>
+      <c r="D48" s="7" t="s">
+        <v>77</v>
       </c>
       <c r="E48" t="s">
         <v>58</v>
       </c>
       <c r="F48" s="7" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>81</v>
+        <v>144</v>
       </c>
       <c r="B49" s="1">
         <v>1</v>
       </c>
       <c r="C49" t="s">
-        <v>104</v>
-      </c>
-      <c r="D49" s="9">
-        <v>5454935</v>
+        <v>76</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>145</v>
       </c>
       <c r="E49" t="s">
         <v>58</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="B50" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C50" t="s">
-        <v>76</v>
-      </c>
-      <c r="D50" s="7" t="s">
-        <v>77</v>
+        <v>66</v>
+      </c>
+      <c r="D50" s="11" t="s">
+        <v>72</v>
       </c>
       <c r="E50" t="s">
         <v>58</v>
       </c>
       <c r="F50" s="7" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>146</v>
+        <v>69</v>
       </c>
       <c r="B51" s="1">
         <v>1</v>
       </c>
       <c r="C51" t="s">
-        <v>76</v>
-      </c>
-      <c r="D51" s="5" t="s">
-        <v>147</v>
+        <v>66</v>
+      </c>
+      <c r="D51" s="11" t="s">
+        <v>67</v>
       </c>
       <c r="E51" t="s">
         <v>58</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="B52" s="1">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C52" t="s">
         <v>66</v>
       </c>
-      <c r="D52" s="11" t="s">
-        <v>72</v>
+      <c r="D52" s="5" t="s">
+        <v>73</v>
       </c>
       <c r="E52" t="s">
         <v>58</v>
       </c>
       <c r="F52" s="7" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="B53" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C53" t="s">
-        <v>66</v>
-      </c>
-      <c r="D53" s="11" t="s">
-        <v>67</v>
+        <v>76</v>
+      </c>
+      <c r="D53" s="5" t="s">
+        <v>135</v>
       </c>
       <c r="E53" t="s">
         <v>58</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>75</v>
+        <v>134</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A54" s="3" t="s">
+        <v>163</v>
       </c>
       <c r="B54" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C54" t="s">
-        <v>66</v>
+        <v>30</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>73</v>
+        <v>166</v>
       </c>
       <c r="E54" t="s">
-        <v>58</v>
-      </c>
-      <c r="F54" s="7" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+      <c r="F54" s="5" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>75</v>
+        <v>164</v>
       </c>
       <c r="B55" s="1">
         <v>2</v>
       </c>
       <c r="C55" t="s">
-        <v>76</v>
+        <v>30</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>136</v>
+        <v>165</v>
       </c>
       <c r="E55" t="s">
-        <v>58</v>
-      </c>
-      <c r="F55" s="7" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+      <c r="F55" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
         <v>168</v>
       </c>
@@ -2190,18 +2287,18 @@
         <v>30</v>
       </c>
       <c r="D56" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="E56" t="s">
+        <v>30</v>
+      </c>
+      <c r="F56" s="5" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
         <v>171</v>
-      </c>
-      <c r="E56" t="s">
-        <v>30</v>
-      </c>
-      <c r="F56" s="5" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>169</v>
       </c>
       <c r="B57" s="1">
         <v>2</v>
@@ -2210,78 +2307,78 @@
         <v>30</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E57" t="s">
         <v>30</v>
       </c>
       <c r="F57" s="5" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A58" s="3" t="s">
-        <v>173</v>
+        <v>89</v>
       </c>
       <c r="B58" s="1">
+        <v>5</v>
+      </c>
+      <c r="C58" t="s">
+        <v>30</v>
+      </c>
+      <c r="D58" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="E58" t="s">
+        <v>30</v>
+      </c>
+      <c r="F58" s="8" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A59" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B59" s="1">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>30</v>
+      </c>
+      <c r="D59" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="E59" t="s">
+        <v>30</v>
+      </c>
+      <c r="F59" s="8" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A60" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="B60" s="1">
         <v>2</v>
       </c>
-      <c r="C58" t="s">
-        <v>30</v>
-      </c>
-      <c r="D58" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="E58" t="s">
-        <v>30</v>
-      </c>
-      <c r="F58" s="5" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>176</v>
-      </c>
-      <c r="B59" s="1">
-        <v>2</v>
-      </c>
-      <c r="C59" t="s">
-        <v>30</v>
-      </c>
-      <c r="D59" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="E59" t="s">
-        <v>30</v>
-      </c>
-      <c r="F59" s="5" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A60" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="B60" s="1">
-        <v>5</v>
-      </c>
       <c r="C60" t="s">
         <v>30</v>
       </c>
       <c r="D60" s="8" t="s">
-        <v>90</v>
+        <v>189</v>
       </c>
       <c r="E60" t="s">
         <v>30</v>
       </c>
       <c r="F60" s="8" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A61" s="3" t="s">
-        <v>88</v>
+        <v>189</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>162</v>
       </c>
       <c r="B61" s="1">
         <v>3</v>
@@ -2290,78 +2387,78 @@
         <v>30</v>
       </c>
       <c r="D61" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E61" t="s">
         <v>30</v>
       </c>
       <c r="F61" s="8" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A62" s="3" t="s">
-        <v>197</v>
+        <v>169</v>
       </c>
       <c r="B62" s="1">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>30</v>
+      </c>
+      <c r="D62" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="E62" t="s">
+        <v>30</v>
+      </c>
+      <c r="F62" s="8" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A63" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B63" s="1">
+        <v>24</v>
+      </c>
+      <c r="C63" t="s">
+        <v>30</v>
+      </c>
+      <c r="D63" t="s">
+        <v>87</v>
+      </c>
+      <c r="E63" t="s">
+        <v>30</v>
+      </c>
+      <c r="F63" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A64" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="B64" s="1">
         <v>2</v>
       </c>
-      <c r="C62" t="s">
-        <v>30</v>
-      </c>
-      <c r="D62" s="8" t="s">
-        <v>198</v>
-      </c>
-      <c r="E62" t="s">
-        <v>30</v>
-      </c>
-      <c r="F62" s="8" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>167</v>
-      </c>
-      <c r="B63" s="1">
-        <v>3</v>
-      </c>
-      <c r="C63" t="s">
-        <v>30</v>
-      </c>
-      <c r="D63" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="E63" t="s">
-        <v>30</v>
-      </c>
-      <c r="F63" s="8" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A64" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="B64" s="1">
-        <v>3</v>
-      </c>
       <c r="C64" t="s">
         <v>30</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>94</v>
+        <v>191</v>
       </c>
       <c r="E64" t="s">
         <v>30</v>
       </c>
       <c r="F64" s="8" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A65" s="3" t="s">
-        <v>149</v>
+        <v>191</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
+        <v>161</v>
       </c>
       <c r="B65" s="1">
         <v>24</v>
@@ -2369,259 +2466,489 @@
       <c r="C65" t="s">
         <v>30</v>
       </c>
-      <c r="D65" t="s">
-        <v>87</v>
+      <c r="D65" s="8" t="s">
+        <v>93</v>
       </c>
       <c r="E65" t="s">
         <v>30</v>
       </c>
-      <c r="F65" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="F65" s="8" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A66" s="3" t="s">
-        <v>199</v>
+        <v>170</v>
       </c>
       <c r="B66" s="1">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="C66" t="s">
         <v>30</v>
       </c>
       <c r="D66" s="8" t="s">
-        <v>200</v>
+        <v>95</v>
       </c>
       <c r="E66" t="s">
         <v>30</v>
       </c>
       <c r="F66" s="8" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>166</v>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A67" s="3" t="s">
+        <v>157</v>
       </c>
       <c r="B67" s="1">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="C67" t="s">
         <v>30</v>
       </c>
       <c r="D67" s="8" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E67" t="s">
         <v>30</v>
       </c>
       <c r="F67" s="8" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A68" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B68" s="1">
+        <v>4</v>
+      </c>
+      <c r="C68" t="s">
+        <v>30</v>
+      </c>
+      <c r="D68" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="E68" t="s">
+        <v>30</v>
+      </c>
+      <c r="F68" s="8" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A69" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="B69" s="1">
+        <v>4</v>
+      </c>
+      <c r="C69" t="s">
+        <v>30</v>
+      </c>
+      <c r="D69" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="E69" t="s">
+        <v>30</v>
+      </c>
+      <c r="F69" s="8" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>148</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C70" t="s">
+        <v>150</v>
+      </c>
+      <c r="D70" t="s">
+        <v>149</v>
+      </c>
+      <c r="E70" t="s">
         <v>175</v>
       </c>
-      <c r="B68" s="1">
-        <v>24</v>
-      </c>
-      <c r="C68" t="s">
-        <v>30</v>
-      </c>
-      <c r="D68" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="E68" t="s">
-        <v>30</v>
-      </c>
-      <c r="F68" s="8" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A69" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="B69" s="1">
-        <v>8</v>
-      </c>
-      <c r="C69" t="s">
-        <v>30</v>
-      </c>
-      <c r="D69" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="E69" t="s">
-        <v>30</v>
-      </c>
-      <c r="F69" s="8" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A70" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="B70" s="1">
-        <v>4</v>
-      </c>
-      <c r="C70" t="s">
-        <v>30</v>
-      </c>
-      <c r="D70" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="E70" t="s">
-        <v>30</v>
-      </c>
-      <c r="F70" s="8" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A71" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="B71" s="1">
-        <v>4</v>
+      <c r="F70" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>179</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>56</v>
       </c>
       <c r="C71" t="s">
-        <v>30</v>
+        <v>123</v>
       </c>
       <c r="D71" s="8" t="s">
-        <v>165</v>
+        <v>182</v>
       </c>
       <c r="E71" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F71" s="8" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>150</v>
+        <v>180</v>
       </c>
       <c r="B72" s="1" t="s">
         <v>56</v>
       </c>
       <c r="C72" t="s">
-        <v>152</v>
-      </c>
-      <c r="D72" t="s">
-        <v>151</v>
+        <v>123</v>
+      </c>
+      <c r="D72" s="8" t="s">
+        <v>183</v>
       </c>
       <c r="E72" t="s">
+        <v>27</v>
+      </c>
+      <c r="F72" s="8" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
         <v>181</v>
-      </c>
-      <c r="F72" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
-        <v>188</v>
       </c>
       <c r="B73" s="1" t="s">
         <v>56</v>
       </c>
       <c r="C73" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D73" s="8" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="E73" t="s">
         <v>27</v>
       </c>
       <c r="F73" s="8" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>189</v>
-      </c>
-      <c r="B74" s="1" t="s">
-        <v>56</v>
+        <v>174</v>
+      </c>
+      <c r="B74" s="1">
+        <v>1</v>
       </c>
       <c r="C74" t="s">
-        <v>124</v>
+        <v>173</v>
       </c>
       <c r="D74" s="8" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="E74" t="s">
-        <v>27</v>
+        <v>173</v>
       </c>
       <c r="F74" s="8" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
-        <v>190</v>
-      </c>
-      <c r="B75" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C75" t="s">
-        <v>124</v>
-      </c>
-      <c r="D75" s="8" t="s">
-        <v>193</v>
-      </c>
-      <c r="E75" t="s">
-        <v>27</v>
-      </c>
-      <c r="F75" s="8" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
-        <v>180</v>
-      </c>
-      <c r="B76" s="1">
-        <v>1</v>
-      </c>
-      <c r="C76" t="s">
-        <v>178</v>
-      </c>
-      <c r="D76" s="8" t="s">
-        <v>214</v>
-      </c>
-      <c r="E76" t="s">
-        <v>178</v>
-      </c>
-      <c r="F76" s="8" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
-        <v>179</v>
-      </c>
-      <c r="B77" s="1">
-        <v>1</v>
-      </c>
-      <c r="C77" t="s">
-        <v>178</v>
-      </c>
-      <c r="D77" s="13" t="s">
-        <v>213</v>
-      </c>
-      <c r="E77" t="s">
-        <v>178</v>
-      </c>
-      <c r="F77" s="13" t="s">
-        <v>213</v>
-      </c>
+        <v>205</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="D75" s="13"/>
+      <c r="F75" s="13"/>
     </row>
   </sheetData>
   <printOptions gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5E2B4AE-7EC3-443B-9505-7740A2597B5A}">
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="82.81640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.7265625" style="14"/>
+    <col min="3" max="3" width="21.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="15" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="B4" s="14">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>207</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>204</v>
+      </c>
+      <c r="E4" t="s">
+        <v>207</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="B5" s="14">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>228</v>
+      </c>
+      <c r="D5" t="s">
+        <v>229</v>
+      </c>
+      <c r="E5" t="s">
+        <v>214</v>
+      </c>
+      <c r="F5" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="B6" s="14">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>213</v>
+      </c>
+      <c r="D6" t="s">
+        <v>213</v>
+      </c>
+      <c r="E6" t="s">
+        <v>214</v>
+      </c>
+      <c r="F6" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="B7" s="14">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>216</v>
+      </c>
+      <c r="D7" t="s">
+        <v>217</v>
+      </c>
+      <c r="E7" t="s">
+        <v>214</v>
+      </c>
+      <c r="F7" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="B8" s="14">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>231</v>
+      </c>
+      <c r="D8" t="s">
+        <v>232</v>
+      </c>
+      <c r="E8" t="s">
+        <v>214</v>
+      </c>
+      <c r="F8" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="B9" s="14">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>234</v>
+      </c>
+      <c r="D9" t="s">
+        <v>235</v>
+      </c>
+      <c r="E9" t="s">
+        <v>214</v>
+      </c>
+      <c r="F9" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="C10" t="s">
+        <v>237</v>
+      </c>
+      <c r="D10" t="s">
+        <v>238</v>
+      </c>
+      <c r="E10" t="s">
+        <v>214</v>
+      </c>
+      <c r="F10" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" s="15" t="s">
+        <v>239</v>
+      </c>
+      <c r="B12" s="16">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="15" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="B16" s="14">
+        <v>1</v>
+      </c>
+      <c r="C16" t="s">
+        <v>207</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>204</v>
+      </c>
+      <c r="E16" t="s">
+        <v>207</v>
+      </c>
+      <c r="F16" s="13" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="B17" s="14">
+        <v>1</v>
+      </c>
+      <c r="C17" t="s">
+        <v>220</v>
+      </c>
+      <c r="D17" t="s">
+        <v>221</v>
+      </c>
+      <c r="E17" t="s">
+        <v>214</v>
+      </c>
+      <c r="F17" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A18" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="C18" t="s">
+        <v>223</v>
+      </c>
+      <c r="D18">
+        <v>16300</v>
+      </c>
+      <c r="E18" t="s">
+        <v>214</v>
+      </c>
+      <c r="F18" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="C19" t="s">
+        <v>225</v>
+      </c>
+      <c r="D19" t="s">
+        <v>226</v>
+      </c>
+      <c r="E19" t="s">
+        <v>214</v>
+      </c>
+      <c r="F19" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" s="15" t="s">
+        <v>240</v>
+      </c>
+      <c r="B21" s="16">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="B22" s="17"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{d546e5e1-5d42-4630-bacd-c69bfdcbd5e8}" enabled="1" method="Standard" siteId="{96ece526-9c7d-48b0-8daf-8b93c90a5d18}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>